<commit_message>
add modification of time spend by module
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1161157069"/>
-        <c:axId val="1288611180"/>
+        <c:axId val="1170378333"/>
+        <c:axId val="1026408693"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1161157069"/>
+        <c:axId val="1170378333"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1288611180"/>
+        <c:crossAx val="1026408693"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1288611180"/>
+        <c:axId val="1026408693"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1161157069"/>
+        <c:crossAx val="1170378333"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="321030192"/>
-        <c:axId val="848962272"/>
+        <c:axId val="613081176"/>
+        <c:axId val="383002026"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="321030192"/>
+        <c:axId val="613081176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="848962272"/>
+        <c:crossAx val="383002026"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="848962272"/>
+        <c:axId val="383002026"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="321030192"/>
+        <c:crossAx val="613081176"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1194,6 +1194,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="7" max="7" width="25.88"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -1323,10 +1326,10 @@
         <v>46192.0</v>
       </c>
       <c r="B6" s="3">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="C6" s="3">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
       <c r="D6" s="3">
         <v>0.0</v>
@@ -1347,17 +1350,25 @@
       <c r="A7" s="5">
         <v>46195.0</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="B7" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F7" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G7" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -1374,7 +1385,7 @@
       </c>
       <c r="G8" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -1391,7 +1402,7 @@
       </c>
       <c r="G9" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -1408,7 +1419,7 @@
       </c>
       <c r="G10" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
@@ -1425,7 +1436,7 @@
       </c>
       <c r="G11" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -1442,7 +1453,7 @@
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
@@ -1459,7 +1470,7 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -1476,7 +1487,7 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
@@ -1493,7 +1504,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
@@ -1510,7 +1521,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17">
@@ -1527,7 +1538,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18">
@@ -1544,7 +1555,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19">
@@ -1561,7 +1572,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
@@ -1578,7 +1589,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21">
@@ -1595,7 +1606,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1658,7 +1669,7 @@
       </c>
       <c r="B2" s="8">
         <f>SUM(Tracker!B2:B21)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -1667,7 +1678,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Tracker!C2:C21)</f>
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -1676,7 +1687,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 23/06 and 24/06
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1170378333"/>
-        <c:axId val="1026408693"/>
+        <c:axId val="1869091880"/>
+        <c:axId val="1253322995"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1170378333"/>
+        <c:axId val="1869091880"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1026408693"/>
+        <c:crossAx val="1253322995"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1026408693"/>
+        <c:axId val="1253322995"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1170378333"/>
+        <c:crossAx val="1869091880"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="613081176"/>
-        <c:axId val="383002026"/>
+        <c:axId val="676318443"/>
+        <c:axId val="30130411"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="613081176"/>
+        <c:axId val="676318443"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="383002026"/>
+        <c:crossAx val="30130411"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="383002026"/>
+        <c:axId val="30130411"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="613081176"/>
+        <c:crossAx val="676318443"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1375,34 +1375,50 @@
       <c r="A8" s="5">
         <v>46196.0</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="B8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2.0</v>
+      </c>
       <c r="F8" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G8" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5">
         <v>46197.0</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="B9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>2.0</v>
+      </c>
       <c r="F9" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G9" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10">
@@ -1419,7 +1435,7 @@
       </c>
       <c r="G10" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
@@ -1436,7 +1452,7 @@
       </c>
       <c r="G11" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
@@ -1453,7 +1469,7 @@
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -1470,7 +1486,7 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14">
@@ -1487,7 +1503,7 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -1504,7 +1520,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16">
@@ -1521,7 +1537,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
@@ -1538,7 +1554,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18">
@@ -1555,7 +1571,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19">
@@ -1572,7 +1588,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20">
@@ -1589,7 +1605,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21">
@@ -1606,7 +1622,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1687,7 +1703,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -1696,7 +1712,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Tracker!E2:E21)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add report of 25/06
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1869091880"/>
-        <c:axId val="1253322995"/>
+        <c:axId val="570876849"/>
+        <c:axId val="1288208155"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1869091880"/>
+        <c:axId val="570876849"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1253322995"/>
+        <c:crossAx val="1288208155"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1253322995"/>
+        <c:axId val="1288208155"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1869091880"/>
+        <c:crossAx val="570876849"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="676318443"/>
-        <c:axId val="30130411"/>
+        <c:axId val="1917749716"/>
+        <c:axId val="307940947"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="676318443"/>
+        <c:axId val="1917749716"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30130411"/>
+        <c:crossAx val="307940947"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30130411"/>
+        <c:axId val="307940947"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="676318443"/>
+        <c:crossAx val="1917749716"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1425,17 +1425,25 @@
       <c r="A10" s="5">
         <v>46198.0</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="B10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1.0</v>
+      </c>
       <c r="F10" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G10" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11">
@@ -1452,7 +1460,7 @@
       </c>
       <c r="G11" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
@@ -1469,7 +1477,7 @@
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13">
@@ -1486,7 +1494,7 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14">
@@ -1503,7 +1511,7 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15">
@@ -1520,7 +1528,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16">
@@ -1537,7 +1545,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17">
@@ -1554,7 +1562,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18">
@@ -1571,7 +1579,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
@@ -1588,7 +1596,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20">
@@ -1605,7 +1613,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21">
@@ -1622,7 +1630,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1703,7 +1711,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -1712,7 +1720,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Tracker!E2:E21)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add report of 26/06
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="570876849"/>
-        <c:axId val="1288208155"/>
+        <c:axId val="913446861"/>
+        <c:axId val="1610320269"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="570876849"/>
+        <c:axId val="913446861"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1288208155"/>
+        <c:crossAx val="1610320269"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1288208155"/>
+        <c:axId val="1610320269"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="570876849"/>
+        <c:crossAx val="913446861"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1917749716"/>
-        <c:axId val="307940947"/>
+        <c:axId val="333083671"/>
+        <c:axId val="110549671"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1917749716"/>
+        <c:axId val="333083671"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="307940947"/>
+        <c:crossAx val="110549671"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="307940947"/>
+        <c:axId val="110549671"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1917749716"/>
+        <c:crossAx val="333083671"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1450,17 +1450,25 @@
       <c r="A11" s="5">
         <v>46199.0</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="B11" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1.0</v>
+      </c>
       <c r="F11" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G11" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
@@ -1477,7 +1485,7 @@
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
@@ -1494,7 +1502,7 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14">
@@ -1511,7 +1519,7 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15">
@@ -1528,7 +1536,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
@@ -1545,7 +1553,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17">
@@ -1562,7 +1570,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18">
@@ -1579,7 +1587,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19">
@@ -1596,7 +1604,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20">
@@ -1613,7 +1621,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21">
@@ -1630,7 +1638,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1711,7 +1719,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -1720,7 +1728,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Tracker!E2:E21)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add report of 29/06
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="913446861"/>
-        <c:axId val="1610320269"/>
+        <c:axId val="1154151333"/>
+        <c:axId val="26086465"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="913446861"/>
+        <c:axId val="1154151333"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1610320269"/>
+        <c:crossAx val="26086465"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1610320269"/>
+        <c:axId val="26086465"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="913446861"/>
+        <c:crossAx val="1154151333"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="333083671"/>
-        <c:axId val="110549671"/>
+        <c:axId val="830603050"/>
+        <c:axId val="2103631261"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="333083671"/>
+        <c:axId val="830603050"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="110549671"/>
+        <c:crossAx val="2103631261"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="110549671"/>
+        <c:axId val="2103631261"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="333083671"/>
+        <c:crossAx val="830603050"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1475,17 +1475,25 @@
       <c r="A12" s="2">
         <v>46202.0</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="B12" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>2.0</v>
+      </c>
       <c r="F12" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G12" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13">
@@ -1502,7 +1510,7 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
@@ -1519,7 +1527,7 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15">
@@ -1536,7 +1544,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16">
@@ -1553,7 +1561,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17">
@@ -1570,7 +1578,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18">
@@ -1587,7 +1595,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19">
@@ -1604,7 +1612,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20">
@@ -1621,7 +1629,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21">
@@ -1638,7 +1646,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1719,7 +1727,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -1728,7 +1736,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Tracker!E2:E21)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add report of 30/06
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1154151333"/>
-        <c:axId val="26086465"/>
+        <c:axId val="908917988"/>
+        <c:axId val="1088699588"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1154151333"/>
+        <c:axId val="908917988"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26086465"/>
+        <c:crossAx val="1088699588"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26086465"/>
+        <c:axId val="1088699588"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1154151333"/>
+        <c:crossAx val="908917988"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="830603050"/>
-        <c:axId val="2103631261"/>
+        <c:axId val="1989612927"/>
+        <c:axId val="727526461"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="830603050"/>
+        <c:axId val="1989612927"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2103631261"/>
+        <c:crossAx val="727526461"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2103631261"/>
+        <c:axId val="727526461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="830603050"/>
+        <c:crossAx val="1989612927"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1500,17 +1500,25 @@
       <c r="A13" s="2">
         <v>46203.0</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
+      <c r="B13" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F13" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G13" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
@@ -1527,7 +1535,7 @@
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15">
@@ -1544,7 +1552,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
@@ -1561,7 +1569,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -1578,7 +1586,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18">
@@ -1595,7 +1603,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19">
@@ -1612,7 +1620,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20">
@@ -1629,7 +1637,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21">
@@ -1646,7 +1654,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1727,7 +1735,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 1/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="908917988"/>
-        <c:axId val="1088699588"/>
+        <c:axId val="1610856301"/>
+        <c:axId val="1124162300"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="908917988"/>
+        <c:axId val="1610856301"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1088699588"/>
+        <c:crossAx val="1124162300"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1088699588"/>
+        <c:axId val="1124162300"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="908917988"/>
+        <c:crossAx val="1610856301"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1989612927"/>
-        <c:axId val="727526461"/>
+        <c:axId val="1948945258"/>
+        <c:axId val="978051608"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1989612927"/>
+        <c:axId val="1948945258"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="727526461"/>
+        <c:crossAx val="978051608"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="727526461"/>
+        <c:axId val="978051608"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1989612927"/>
+        <c:crossAx val="1948945258"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1525,17 +1525,25 @@
       <c r="A14" s="2">
         <v>46204.0</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+      <c r="B14" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>4.0</v>
+      </c>
       <c r="F14" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G14" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15">
@@ -1552,7 +1560,7 @@
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">
@@ -1569,7 +1577,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17">
@@ -1586,7 +1594,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18">
@@ -1603,7 +1611,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19">
@@ -1620,7 +1628,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20">
@@ -1637,7 +1645,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21">
@@ -1654,7 +1662,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1735,7 +1743,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -1744,7 +1752,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Tracker!E2:E21)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add report of 2/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1610856301"/>
-        <c:axId val="1124162300"/>
+        <c:axId val="1326107157"/>
+        <c:axId val="806604917"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1610856301"/>
+        <c:axId val="1326107157"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1124162300"/>
+        <c:crossAx val="806604917"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1124162300"/>
+        <c:axId val="806604917"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1610856301"/>
+        <c:crossAx val="1326107157"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1948945258"/>
-        <c:axId val="978051608"/>
+        <c:axId val="580496881"/>
+        <c:axId val="1493340344"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1948945258"/>
+        <c:axId val="580496881"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="978051608"/>
+        <c:crossAx val="1493340344"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="978051608"/>
+        <c:axId val="1493340344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1948945258"/>
+        <c:crossAx val="580496881"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1550,17 +1550,25 @@
       <c r="A15" s="2">
         <v>46205.0</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
+      <c r="B15" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>2.0</v>
+      </c>
       <c r="F15" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G15" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16">
@@ -1577,7 +1585,7 @@
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17">
@@ -1594,7 +1602,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18">
@@ -1611,7 +1619,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19">
@@ -1628,7 +1636,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20">
@@ -1645,7 +1653,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21">
@@ -1662,7 +1670,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1743,7 +1751,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -1752,7 +1760,7 @@
       </c>
       <c r="B5" s="8">
         <f>SUM(Tracker!E2:E21)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add report of 3/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1326107157"/>
-        <c:axId val="806604917"/>
+        <c:axId val="1217743808"/>
+        <c:axId val="1699721842"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1326107157"/>
+        <c:axId val="1217743808"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="806604917"/>
+        <c:crossAx val="1699721842"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="806604917"/>
+        <c:axId val="1699721842"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1326107157"/>
+        <c:crossAx val="1217743808"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="580496881"/>
-        <c:axId val="1493340344"/>
+        <c:axId val="1295241353"/>
+        <c:axId val="516833084"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="580496881"/>
+        <c:axId val="1295241353"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1493340344"/>
+        <c:crossAx val="516833084"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1493340344"/>
+        <c:axId val="516833084"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="580496881"/>
+        <c:crossAx val="1295241353"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1575,17 +1575,25 @@
       <c r="A16" s="2">
         <v>46206.0</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="B16" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F16" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G16" s="4">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17">
@@ -1602,7 +1610,7 @@
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18">
@@ -1619,7 +1627,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19">
@@ -1636,7 +1644,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20">
@@ -1653,7 +1661,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21">
@@ -1670,7 +1678,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1751,7 +1759,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 6/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1217743808"/>
-        <c:axId val="1699721842"/>
+        <c:axId val="1083174171"/>
+        <c:axId val="1710629798"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1217743808"/>
+        <c:axId val="1083174171"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1699721842"/>
+        <c:crossAx val="1710629798"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1699721842"/>
+        <c:axId val="1710629798"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1217743808"/>
+        <c:crossAx val="1083174171"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1295241353"/>
-        <c:axId val="516833084"/>
+        <c:axId val="327824604"/>
+        <c:axId val="1263839798"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1295241353"/>
+        <c:axId val="327824604"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="516833084"/>
+        <c:crossAx val="1263839798"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="516833084"/>
+        <c:axId val="1263839798"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1295241353"/>
+        <c:crossAx val="327824604"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1600,17 +1600,25 @@
       <c r="A17" s="5">
         <v>46209.0</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="B17" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F17" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G17" s="4">
         <f t="shared" si="2"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18">
@@ -1627,7 +1635,7 @@
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19">
@@ -1644,7 +1652,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20">
@@ -1661,7 +1669,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21">
@@ -1678,7 +1686,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1759,7 +1767,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add checkPensioner to search trough a database in thomas/db/ 20 pensioners of each class and look if they have a own page on prosocour website
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1083174171"/>
-        <c:axId val="1710629798"/>
+        <c:axId val="1050866924"/>
+        <c:axId val="125182429"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1083174171"/>
+        <c:axId val="1050866924"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1710629798"/>
+        <c:crossAx val="125182429"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1710629798"/>
+        <c:axId val="125182429"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1083174171"/>
+        <c:crossAx val="1050866924"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="327824604"/>
-        <c:axId val="1263839798"/>
+        <c:axId val="605674999"/>
+        <c:axId val="1016843112"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="327824604"/>
+        <c:axId val="605674999"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1263839798"/>
+        <c:crossAx val="1016843112"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1263839798"/>
+        <c:axId val="1016843112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="327824604"/>
+        <c:crossAx val="605674999"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1625,17 +1625,25 @@
       <c r="A18" s="5">
         <v>46210.0</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="B18" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F18" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19">
@@ -1652,7 +1660,7 @@
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20">
@@ -1669,7 +1677,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21">
@@ -1686,7 +1694,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1767,7 +1775,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 8/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1050866924"/>
-        <c:axId val="125182429"/>
+        <c:axId val="910203626"/>
+        <c:axId val="1247377169"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1050866924"/>
+        <c:axId val="910203626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="125182429"/>
+        <c:crossAx val="1247377169"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="125182429"/>
+        <c:axId val="1247377169"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1050866924"/>
+        <c:crossAx val="910203626"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="605674999"/>
-        <c:axId val="1016843112"/>
+        <c:axId val="189045745"/>
+        <c:axId val="1480013300"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="605674999"/>
+        <c:axId val="189045745"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1016843112"/>
+        <c:crossAx val="1480013300"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1016843112"/>
+        <c:axId val="1480013300"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="605674999"/>
+        <c:crossAx val="189045745"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1650,17 +1650,25 @@
       <c r="A19" s="5">
         <v>46211.0</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="B19" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F19" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G19" s="4">
         <f t="shared" si="2"/>
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
@@ -1677,7 +1685,7 @@
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21">
@@ -1694,7 +1702,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1775,7 +1783,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 9/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="910203626"/>
-        <c:axId val="1247377169"/>
+        <c:axId val="1481387828"/>
+        <c:axId val="1411204425"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="910203626"/>
+        <c:axId val="1481387828"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1247377169"/>
+        <c:crossAx val="1411204425"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1247377169"/>
+        <c:axId val="1411204425"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="910203626"/>
+        <c:crossAx val="1481387828"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="189045745"/>
-        <c:axId val="1480013300"/>
+        <c:axId val="1264059244"/>
+        <c:axId val="64965278"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="189045745"/>
+        <c:axId val="1264059244"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480013300"/>
+        <c:crossAx val="64965278"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1480013300"/>
+        <c:axId val="64965278"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="189045745"/>
+        <c:crossAx val="1264059244"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1675,17 +1675,25 @@
       <c r="A20" s="5">
         <v>46212.0</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
+      <c r="B20" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F20" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G20" s="4">
         <f t="shared" si="2"/>
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21">
@@ -1702,7 +1710,7 @@
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1783,7 +1791,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 10/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -489,11 +489,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1481387828"/>
-        <c:axId val="1411204425"/>
+        <c:axId val="437838023"/>
+        <c:axId val="1216628383"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1481387828"/>
+        <c:axId val="437838023"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +549,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1411204425"/>
+        <c:crossAx val="1216628383"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1411204425"/>
+        <c:axId val="1216628383"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1481387828"/>
+        <c:crossAx val="437838023"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +721,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1264059244"/>
-        <c:axId val="64965278"/>
+        <c:axId val="277876040"/>
+        <c:axId val="1201840044"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1264059244"/>
+        <c:axId val="277876040"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +781,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64965278"/>
+        <c:crossAx val="1201840044"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64965278"/>
+        <c:axId val="1201840044"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1264059244"/>
+        <c:crossAx val="277876040"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1700,17 +1700,25 @@
       <c r="A21" s="5">
         <v>46213.0</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
+      <c r="B21" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="E21" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F21" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G21" s="4">
         <f t="shared" si="2"/>
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1791,7 +1799,7 @@
       </c>
       <c r="B4" s="8">
         <f>SUM(Tracker!D2:D21)</f>
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Add report of 27/07, modification of checkPensioner to limit insertion on database of authority links by setting a variable
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -13,7 +13,25 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Temps Total</t>
+  </si>
+  <si>
+    <t>Module 1</t>
+  </si>
+  <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
+  </si>
   <si>
     <t>Date</t>
   </si>
@@ -38,24 +56,6 @@
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
   </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Temps Total</t>
-  </si>
-  <si>
-    <t>Module 1</t>
-  </si>
-  <si>
-    <t>Module 2</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
-  </si>
 </sst>
 </file>
 
@@ -68,6 +68,11 @@
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -86,13 +91,8 @@
       <color theme="1"/>
       <name val="Montserrat"/>
     </font>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -111,6 +111,12 @@
         <bgColor rgb="FFB6D7A8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -118,30 +124,33 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -197,8 +206,13 @@
       <border/>
     </dxf>
   </dxfs>
-  <tableStyles count="1">
+  <tableStyles count="2">
     <tableStyle count="3" pivot="0" name="Tracker-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+    </tableStyle>
+    <tableStyle count="3" pivot="0" name="Tracker-style 2">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -489,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="437838023"/>
-        <c:axId val="1216628383"/>
+        <c:axId val="2014838202"/>
+        <c:axId val="1169376268"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="437838023"/>
+        <c:axId val="2014838202"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1216628383"/>
+        <c:crossAx val="1169376268"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1216628383"/>
+        <c:axId val="1169376268"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -629,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="437838023"/>
+        <c:crossAx val="2014838202"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -721,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="277876040"/>
-        <c:axId val="1201840044"/>
+        <c:axId val="89694806"/>
+        <c:axId val="1911584662"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="277876040"/>
+        <c:axId val="89694806"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -781,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1201840044"/>
+        <c:crossAx val="1911584662"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1201840044"/>
+        <c:axId val="1911584662"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -861,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="277876040"/>
+        <c:crossAx val="89694806"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -991,6 +1005,21 @@
     <tableColumn name="Progression Cumulée" id="7"/>
   </tableColumns>
   <tableStyleInfo name="Tracker-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="I1:O21" displayName="Table_2" name="Table_2" id="2">
+  <tableColumns count="7">
+    <tableColumn name="Date" id="1"/>
+    <tableColumn name="Découpe" id="2"/>
+    <tableColumn name="Extraction" id="3"/>
+    <tableColumn name="Backoffice" id="4"/>
+    <tableColumn name="FrontOffice" id="5"/>
+    <tableColumn name="Total Jour" id="6"/>
+    <tableColumn name="Progression Cumulée" id="7"/>
+  </tableColumns>
+  <tableStyleInfo name="Tracker-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -1199,543 +1228,876 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>46188.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5">
         <v>4.0</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="5">
         <v>3.0</v>
       </c>
-      <c r="D2" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E2" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F2" s="4">
+      <c r="D2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F2" s="6">
         <f t="shared" ref="F2:F21" si="1">SUM(B2:E2)</f>
         <v>7</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="6">
         <f t="shared" ref="G2:G21" si="2">SUM($F$2:F2)</f>
         <v>7</v>
       </c>
+      <c r="I2" s="4">
+        <v>46230.0</v>
+      </c>
+      <c r="J2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L2" s="5">
+        <v>6.0</v>
+      </c>
+      <c r="M2" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="N2" s="6">
+        <f t="shared" ref="N2:N21" si="3">SUM(J2:M2)</f>
+        <v>7</v>
+      </c>
+      <c r="O2" s="6">
+        <f t="shared" ref="O2:O21" si="4">SUM($N$2:N2)</f>
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>46189.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>2.0</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="5">
         <v>5.0</v>
       </c>
-      <c r="D3" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F3" s="4">
+      <c r="D3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="6">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
+      <c r="I3" s="4">
+        <v>46231.0</v>
+      </c>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O3" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>46190.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>2.0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="5">
         <v>5.0</v>
       </c>
-      <c r="D4" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F4" s="4">
+      <c r="D4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="6">
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
+      <c r="I4" s="4">
+        <v>46232.0</v>
+      </c>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O4" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>46191.0</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>4.0</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="5">
         <v>3.0</v>
       </c>
-      <c r="D5" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F5" s="4">
+      <c r="D5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="6">
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
+      <c r="I5" s="4">
+        <v>46233.0</v>
+      </c>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
+      <c r="A6" s="4">
         <v>46192.0</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="5">
         <v>1.0</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="5">
         <v>6.0</v>
       </c>
-      <c r="D6" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F6" s="4">
+      <c r="D6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="6">
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
+      <c r="I6" s="4">
+        <v>46234.0</v>
+      </c>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5">
+      <c r="A7" s="7">
         <v>46195.0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="5">
         <v>3.0</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="5">
         <v>3.0</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="5">
         <v>1.0</v>
       </c>
-      <c r="E7" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F7" s="4">
+      <c r="E7" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="6">
         <f t="shared" si="2"/>
         <v>42</v>
       </c>
+      <c r="I7" s="7">
+        <v>46237.0</v>
+      </c>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5">
+      <c r="A8" s="7">
         <v>46196.0</v>
       </c>
-      <c r="B8" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C8" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D8" s="3">
+      <c r="B8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="5">
         <v>5.0</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="5">
         <v>2.0</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="6">
         <f t="shared" si="2"/>
         <v>49</v>
       </c>
+      <c r="I8" s="7">
+        <v>46238.0</v>
+      </c>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O8" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5">
+      <c r="A9" s="7">
         <v>46197.0</v>
       </c>
-      <c r="B9" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C9" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D9" s="3">
+      <c r="B9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="5">
         <v>5.0</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="5">
         <v>2.0</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="6">
         <f t="shared" si="2"/>
         <v>56</v>
       </c>
+      <c r="I9" s="7">
+        <v>46239.0</v>
+      </c>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O9" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5">
+      <c r="A10" s="7">
         <v>46198.0</v>
       </c>
-      <c r="B10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D10" s="3">
+      <c r="B10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="5">
         <v>6.0</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="5">
         <v>1.0</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="6">
         <f t="shared" si="2"/>
         <v>63</v>
       </c>
+      <c r="I10" s="7">
+        <v>46240.0</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O10" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5">
+      <c r="A11" s="7">
         <v>46199.0</v>
       </c>
-      <c r="B11" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C11" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D11" s="3">
+      <c r="B11" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="5">
         <v>6.0</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="5">
         <v>1.0</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="6">
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
+      <c r="I11" s="7">
+        <v>46241.0</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O11" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2">
+      <c r="A12" s="4">
         <v>46202.0</v>
       </c>
-      <c r="B12" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D12" s="3">
+      <c r="B12" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="5">
         <v>5.0</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="5">
         <v>2.0</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="6">
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
+      <c r="I12" s="4">
+        <v>46244.0</v>
+      </c>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O12" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2">
+      <c r="A13" s="4">
         <v>46203.0</v>
       </c>
-      <c r="B13" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C13" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D13" s="3">
+      <c r="B13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="5">
         <v>7.0</v>
       </c>
-      <c r="E13" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F13" s="4">
+      <c r="E13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F13" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="6">
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
+      <c r="I13" s="4">
+        <v>46245.0</v>
+      </c>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O13" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2">
+      <c r="A14" s="4">
         <v>46204.0</v>
       </c>
-      <c r="B14" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D14" s="3">
+      <c r="B14" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="5">
         <v>3.0</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="5">
         <v>4.0</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="6">
         <f t="shared" si="2"/>
         <v>91</v>
       </c>
+      <c r="I14" s="4">
+        <v>46246.0</v>
+      </c>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O14" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2">
+      <c r="A15" s="4">
         <v>46205.0</v>
       </c>
-      <c r="B15" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C15" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D15" s="3">
+      <c r="B15" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D15" s="5">
         <v>5.0</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="5">
         <v>2.0</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="6">
         <f t="shared" si="2"/>
         <v>98</v>
       </c>
+      <c r="I15" s="4">
+        <v>46247.0</v>
+      </c>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O15" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2">
+      <c r="A16" s="4">
         <v>46206.0</v>
       </c>
-      <c r="B16" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C16" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D16" s="3">
+      <c r="B16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D16" s="5">
         <v>7.0</v>
       </c>
-      <c r="E16" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F16" s="4">
+      <c r="E16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F16" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="6">
         <f t="shared" si="2"/>
         <v>105</v>
       </c>
+      <c r="I16" s="4">
+        <v>46248.0</v>
+      </c>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O16" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5">
+      <c r="A17" s="7">
         <v>46209.0</v>
       </c>
-      <c r="B17" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C17" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D17" s="3">
+      <c r="B17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D17" s="5">
         <v>7.0</v>
       </c>
-      <c r="E17" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F17" s="4">
+      <c r="E17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F17" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="6">
         <f t="shared" si="2"/>
         <v>112</v>
       </c>
+      <c r="I17" s="4">
+        <v>46251.0</v>
+      </c>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O17" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5">
+      <c r="A18" s="7">
         <v>46210.0</v>
       </c>
-      <c r="B18" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C18" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D18" s="3">
+      <c r="B18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D18" s="5">
         <v>7.0</v>
       </c>
-      <c r="E18" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F18" s="4">
+      <c r="E18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F18" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="6">
         <f t="shared" si="2"/>
         <v>119</v>
       </c>
+      <c r="I18" s="4">
+        <v>46252.0</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O18" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5">
+      <c r="A19" s="7">
         <v>46211.0</v>
       </c>
-      <c r="B19" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C19" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D19" s="3">
+      <c r="B19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D19" s="5">
         <v>7.0</v>
       </c>
-      <c r="E19" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F19" s="4">
+      <c r="E19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F19" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="6">
         <f t="shared" si="2"/>
         <v>126</v>
       </c>
+      <c r="I19" s="4">
+        <v>46253.0</v>
+      </c>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O19" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5">
+      <c r="A20" s="7">
         <v>46212.0</v>
       </c>
-      <c r="B20" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C20" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D20" s="3">
+      <c r="B20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D20" s="5">
         <v>7.0</v>
       </c>
-      <c r="E20" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F20" s="4">
+      <c r="E20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F20" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="6">
         <f t="shared" si="2"/>
         <v>133</v>
       </c>
+      <c r="I20" s="4">
+        <v>46254.0</v>
+      </c>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O20" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5">
+      <c r="A21" s="7">
         <v>46213.0</v>
       </c>
-      <c r="B21" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="C21" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D21" s="3">
+      <c r="B21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D21" s="5">
         <v>7.0</v>
       </c>
-      <c r="E21" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="F21" s="4">
+      <c r="E21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F21" s="6">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="6">
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
+      <c r="I21" s="4">
+        <v>46255.0</v>
+      </c>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O21" s="6">
+        <f t="shared" si="4"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="I22" s="9"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F21">
+  <conditionalFormatting sqref="F2:F21 N2:N21">
     <cfRule type="cellIs" dxfId="4" priority="1" stopIfTrue="1" operator="greaterThan">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="B2:E21">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="B2:E21 J2:M21">
       <formula1>0.0</formula1>
       <formula2>7.0</formula2>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1748,8 +2110,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="6" t="s">
-        <v>7</v>
+      <c r="B2" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1768,45 +2130,45 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>9</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="8">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="8">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="8">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="8">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 28/07, add global variables to limit permutation search, adjustment of permutation scores capped at 0.25 and floored at 0.10
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,15 +24,6 @@
     <t>Module 1</t>
   </si>
   <si>
-    <t>Module 2</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -52,6 +43,15 @@
   </si>
   <si>
     <t>Progression Cumulée</t>
+  </si>
+  <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,10 +131,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="2014838202"/>
-        <c:axId val="1169376268"/>
+        <c:axId val="293185762"/>
+        <c:axId val="1336379256"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2014838202"/>
+        <c:axId val="293185762"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1169376268"/>
+        <c:crossAx val="1336379256"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1169376268"/>
+        <c:axId val="1336379256"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2014838202"/>
+        <c:crossAx val="293185762"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="89694806"/>
-        <c:axId val="1911584662"/>
+        <c:axId val="652911197"/>
+        <c:axId val="724718212"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="89694806"/>
+        <c:axId val="652911197"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1911584662"/>
+        <c:crossAx val="724718212"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1911584662"/>
+        <c:axId val="724718212"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89694806"/>
+        <c:crossAx val="652911197"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1228,47 +1228,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -1346,17 +1346,25 @@
       <c r="I3" s="4">
         <v>46231.0</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
+      <c r="J3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L3" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M3" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N3" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O3" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -1396,7 +1404,7 @@
       </c>
       <c r="O4" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -1436,7 +1444,7 @@
       </c>
       <c r="O5" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -1476,7 +1484,7 @@
       </c>
       <c r="O6" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1516,7 +1524,7 @@
       </c>
       <c r="O7" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -1556,7 +1564,7 @@
       </c>
       <c r="O8" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1596,7 +1604,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -1636,7 +1644,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -1676,7 +1684,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -1716,7 +1724,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -1756,7 +1764,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -1796,7 +1804,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -1836,7 +1844,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -1876,7 +1884,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -1916,7 +1924,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -1956,7 +1964,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
@@ -1996,7 +2004,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20">
@@ -2036,7 +2044,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -2076,7 +2084,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -2141,34 +2149,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 29/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,6 +24,15 @@
     <t>Module 1</t>
   </si>
   <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -43,15 +52,6 @@
   </si>
   <si>
     <t>Progression Cumulée</t>
-  </si>
-  <si>
-    <t>Module 2</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,10 +131,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="293185762"/>
-        <c:axId val="1336379256"/>
+        <c:axId val="929079757"/>
+        <c:axId val="1574839078"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="293185762"/>
+        <c:axId val="929079757"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1336379256"/>
+        <c:crossAx val="1574839078"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1336379256"/>
+        <c:axId val="1574839078"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="293185762"/>
+        <c:crossAx val="929079757"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="652911197"/>
-        <c:axId val="724718212"/>
+        <c:axId val="71426251"/>
+        <c:axId val="307015205"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="652911197"/>
+        <c:axId val="71426251"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="724718212"/>
+        <c:crossAx val="307015205"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="724718212"/>
+        <c:axId val="307015205"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="652911197"/>
+        <c:crossAx val="71426251"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1228,47 +1228,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" s="2" t="s">
+      <c r="E1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="2" t="s">
+      <c r="J1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -1394,17 +1394,25 @@
       <c r="I4" s="4">
         <v>46232.0</v>
       </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
+      <c r="J4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L4" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M4" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N4" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O4" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -1444,7 +1452,7 @@
       </c>
       <c r="O5" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -1484,7 +1492,7 @@
       </c>
       <c r="O6" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1524,7 +1532,7 @@
       </c>
       <c r="O7" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1564,7 +1572,7 @@
       </c>
       <c r="O8" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1604,7 +1612,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1644,7 +1652,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
@@ -1684,7 +1692,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -1724,7 +1732,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
@@ -1764,7 +1772,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
@@ -1804,7 +1812,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -1844,7 +1852,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16">
@@ -1884,7 +1892,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
@@ -1924,7 +1932,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -1964,7 +1972,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -2004,7 +2012,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20">
@@ -2044,7 +2052,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -2084,7 +2092,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
@@ -2149,34 +2157,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 30/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="929079757"/>
-        <c:axId val="1574839078"/>
+        <c:axId val="264451850"/>
+        <c:axId val="778385490"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="929079757"/>
+        <c:axId val="264451850"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1574839078"/>
+        <c:crossAx val="778385490"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1574839078"/>
+        <c:axId val="778385490"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="929079757"/>
+        <c:crossAx val="264451850"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="71426251"/>
-        <c:axId val="307015205"/>
+        <c:axId val="507852499"/>
+        <c:axId val="163785281"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="71426251"/>
+        <c:axId val="507852499"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="307015205"/>
+        <c:crossAx val="163785281"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="307015205"/>
+        <c:axId val="163785281"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71426251"/>
+        <c:crossAx val="507852499"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1442,17 +1442,25 @@
       <c r="I5" s="4">
         <v>46233.0</v>
       </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
+      <c r="J5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L5" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M5" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N5" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O5" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
@@ -1492,7 +1500,7 @@
       </c>
       <c r="O6" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -1532,7 +1540,7 @@
       </c>
       <c r="O7" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -1572,7 +1580,7 @@
       </c>
       <c r="O8" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -1612,7 +1620,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -1652,7 +1660,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -1692,7 +1700,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -1732,7 +1740,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
@@ -1772,7 +1780,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -1812,7 +1820,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -1852,7 +1860,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
@@ -1892,7 +1900,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -1919,7 +1927,7 @@
         <f t="shared" si="2"/>
         <v>112</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="7">
         <v>46251.0</v>
       </c>
       <c r="J17" s="5"/>
@@ -1932,7 +1940,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18">
@@ -1959,7 +1967,7 @@
         <f t="shared" si="2"/>
         <v>119</v>
       </c>
-      <c r="I18" s="4">
+      <c r="I18" s="7">
         <v>46252.0</v>
       </c>
       <c r="J18" s="5"/>
@@ -1972,7 +1980,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19">
@@ -1999,7 +2007,7 @@
         <f t="shared" si="2"/>
         <v>126</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="7">
         <v>46253.0</v>
       </c>
       <c r="J19" s="5"/>
@@ -2012,7 +2020,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20">
@@ -2039,7 +2047,7 @@
         <f t="shared" si="2"/>
         <v>133</v>
       </c>
-      <c r="I20" s="4">
+      <c r="I20" s="7">
         <v>46254.0</v>
       </c>
       <c r="J20" s="5"/>
@@ -2052,7 +2060,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21">
@@ -2079,7 +2087,7 @@
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
-      <c r="I21" s="4">
+      <c r="I21" s="7">
         <v>46255.0</v>
       </c>
       <c r="J21" s="5"/>
@@ -2092,7 +2100,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Add report of 31/07
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,15 +24,6 @@
     <t>Module 1</t>
   </si>
   <si>
-    <t>Module 2</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -40,6 +31,9 @@
   </si>
   <si>
     <t>Extraction</t>
+  </si>
+  <si>
+    <t>Module 2</t>
   </si>
   <si>
     <t>Backoffice</t>
@@ -52,6 +46,12 @@
   </si>
   <si>
     <t>Progression Cumulée</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,10 +131,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -145,11 +145,11 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="264451850"/>
-        <c:axId val="778385490"/>
+        <c:axId val="95903124"/>
+        <c:axId val="1330655882"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="264451850"/>
+        <c:axId val="95903124"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="778385490"/>
+        <c:crossAx val="1330655882"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="778385490"/>
+        <c:axId val="1330655882"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="264451850"/>
+        <c:crossAx val="95903124"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="507852499"/>
-        <c:axId val="163785281"/>
+        <c:axId val="284198581"/>
+        <c:axId val="1791739060"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="507852499"/>
+        <c:axId val="284198581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="163785281"/>
+        <c:crossAx val="1791739060"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="163785281"/>
+        <c:axId val="1791739060"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="507852499"/>
+        <c:crossAx val="284198581"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1228,47 +1228,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="I1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -1490,17 +1490,25 @@
       <c r="I6" s="4">
         <v>46234.0</v>
       </c>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="J6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L6" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M6" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N6" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O6" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -1540,7 +1548,7 @@
       </c>
       <c r="O7" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -1580,7 +1588,7 @@
       </c>
       <c r="O8" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
@@ -1620,7 +1628,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -1660,7 +1668,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11">
@@ -1700,7 +1708,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -1740,7 +1748,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
@@ -1780,7 +1788,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14">
@@ -1820,7 +1828,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
@@ -1860,7 +1868,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16">
@@ -1900,7 +1908,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -1940,7 +1948,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -1980,7 +1988,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
@@ -2020,7 +2028,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20">
@@ -2060,7 +2068,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21">
@@ -2100,11 +2108,11 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22">
-      <c r="I22" s="9"/>
+      <c r="I22" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F21 N2:N21">
@@ -2134,7 +2142,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2165,34 +2173,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 03/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,16 +24,22 @@
     <t>Module 1</t>
   </si>
   <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
     <t>Découpe</t>
   </si>
   <si>
-    <t>Extraction</t>
+    <t>Module 4</t>
   </si>
   <si>
-    <t>Module 2</t>
+    <t>Extraction</t>
   </si>
   <si>
     <t>Backoffice</t>
@@ -46,12 +52,6 @@
   </si>
   <si>
     <t>Progression Cumulée</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,10 +131,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="95903124"/>
-        <c:axId val="1330655882"/>
+        <c:axId val="298379645"/>
+        <c:axId val="464967191"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95903124"/>
+        <c:axId val="298379645"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1330655882"/>
+        <c:crossAx val="464967191"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1330655882"/>
+        <c:axId val="464967191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95903124"/>
+        <c:crossAx val="298379645"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="284198581"/>
-        <c:axId val="1791739060"/>
+        <c:axId val="1746623310"/>
+        <c:axId val="374978351"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="284198581"/>
+        <c:axId val="1746623310"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1791739060"/>
+        <c:crossAx val="374978351"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1791739060"/>
+        <c:axId val="374978351"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="284198581"/>
+        <c:crossAx val="1746623310"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1228,47 +1228,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="2" t="s">
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -1538,17 +1538,25 @@
       <c r="I7" s="7">
         <v>46237.0</v>
       </c>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="J7" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L7" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M7" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N7" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O7" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -1588,7 +1596,7 @@
       </c>
       <c r="O8" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -1628,7 +1636,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -1668,7 +1676,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
@@ -1708,7 +1716,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -1748,7 +1756,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
@@ -1788,7 +1796,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -1828,7 +1836,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
@@ -1868,7 +1876,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
@@ -1908,7 +1916,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17">
@@ -1948,7 +1956,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18">
@@ -1988,7 +1996,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19">
@@ -2028,7 +2036,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
@@ -2068,7 +2076,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21">
@@ -2108,7 +2116,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22">
@@ -2173,34 +2181,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 04/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -27,16 +27,16 @@
     <t>Module 2</t>
   </si>
   <si>
+    <t>Date</t>
+  </si>
+  <si>
     <t>Module 3</t>
   </si>
   <si>
-    <t>Date</t>
+    <t>Module 4</t>
   </si>
   <si>
     <t>Découpe</t>
-  </si>
-  <si>
-    <t>Module 4</t>
   </si>
   <si>
     <t>Extraction</t>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="298379645"/>
-        <c:axId val="464967191"/>
+        <c:axId val="497528272"/>
+        <c:axId val="1353082469"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="298379645"/>
+        <c:axId val="497528272"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="464967191"/>
+        <c:crossAx val="1353082469"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="464967191"/>
+        <c:axId val="1353082469"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="298379645"/>
+        <c:crossAx val="497528272"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1746623310"/>
-        <c:axId val="374978351"/>
+        <c:axId val="1480671581"/>
+        <c:axId val="927520650"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1746623310"/>
+        <c:axId val="1480671581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="374978351"/>
+        <c:crossAx val="927520650"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="374978351"/>
+        <c:axId val="927520650"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1746623310"/>
+        <c:crossAx val="1480671581"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1229,10 +1229,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>8</v>
@@ -1250,10 +1250,10 @@
         <v>12</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>8</v>
@@ -1586,17 +1586,25 @@
       <c r="I8" s="7">
         <v>46238.0</v>
       </c>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+      <c r="J8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L8" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M8" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N8" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O8" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9">
@@ -1636,7 +1644,7 @@
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
@@ -1676,7 +1684,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11">
@@ -1716,7 +1724,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -1756,7 +1764,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
@@ -1796,7 +1804,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14">
@@ -1836,7 +1844,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
@@ -1876,7 +1884,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
@@ -1916,7 +1924,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
@@ -1956,7 +1964,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18">
@@ -1996,7 +2004,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19">
@@ -2036,7 +2044,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20">
@@ -2076,7 +2084,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21">
@@ -2116,7 +2124,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
@@ -2197,7 +2205,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
@@ -2206,7 +2214,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>

</xml_diff>

<commit_message>
Add report of 05/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>Module</t>
   </si>
@@ -25,9 +25,6 @@
   </si>
   <si>
     <t>Module 2</t>
-  </si>
-  <si>
-    <t>Date</t>
   </si>
   <si>
     <t>Module 3</t>
@@ -52,6 +49,9 @@
   </si>
   <si>
     <t>Progression Cumulée</t>
+  </si>
+  <si>
+    <t>Date</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -145,11 +145,11 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="497528272"/>
-        <c:axId val="1353082469"/>
+        <c:axId val="1627451947"/>
+        <c:axId val="2076279430"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="497528272"/>
+        <c:axId val="1627451947"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1353082469"/>
+        <c:crossAx val="2076279430"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1353082469"/>
+        <c:axId val="2076279430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="497528272"/>
+        <c:crossAx val="1627451947"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1480671581"/>
-        <c:axId val="927520650"/>
+        <c:axId val="1414164693"/>
+        <c:axId val="1405783839"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1480671581"/>
+        <c:axId val="1414164693"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="927520650"/>
+        <c:crossAx val="1405783839"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="927520650"/>
+        <c:axId val="1405783839"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1480671581"/>
+        <c:crossAx val="1414164693"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -994,17 +994,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G21" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A1:G21" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="7">
-    <tableColumn name="Date" id="1"/>
-    <tableColumn name="Découpe" id="2"/>
-    <tableColumn name="Extraction" id="3"/>
-    <tableColumn name="Backoffice" id="4"/>
-    <tableColumn name="FrontOffice" id="5"/>
-    <tableColumn name="Total Jour" id="6"/>
-    <tableColumn name="Progression Cumulée" id="7"/>
+    <tableColumn name="Column1" id="1"/>
+    <tableColumn name="Column2" id="2"/>
+    <tableColumn name="Column3" id="3"/>
+    <tableColumn name="Column4" id="4"/>
+    <tableColumn name="Column5" id="5"/>
+    <tableColumn name="Column6" id="6"/>
+    <tableColumn name="Column7" id="7"/>
   </tableColumns>
   <tableStyleInfo name="Tracker-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <extLst>
+    <ext uri="GoogleSheetsCustomDataVersion1">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" headerRowCount="1"/>
+    </ext>
+  </extLst>
 </table>
 </file>
 
@@ -1228,47 +1233,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>4</v>
+      <c r="A1" s="3">
+        <v>0.0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>4</v>
-      </c>
       <c r="J1" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -1634,17 +1639,25 @@
       <c r="I9" s="7">
         <v>46239.0</v>
       </c>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="J9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L9" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M9" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N9" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O9" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10">
@@ -1684,7 +1697,7 @@
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
@@ -1724,7 +1737,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
@@ -1764,7 +1777,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -1804,7 +1817,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14">
@@ -1844,7 +1857,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -1884,7 +1897,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16">
@@ -1924,7 +1937,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
@@ -1964,7 +1977,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18">
@@ -2004,7 +2017,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19">
@@ -2044,7 +2057,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20">
@@ -2084,7 +2097,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21">
@@ -2124,11 +2137,11 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22">
-      <c r="I22" s="8"/>
+      <c r="I22" s="9"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F21 N2:N21">
@@ -2158,7 +2171,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2205,7 +2218,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
@@ -2214,7 +2227,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>

</xml_diff>

<commit_message>
Add report of 06/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1627451947"/>
-        <c:axId val="2076279430"/>
+        <c:axId val="1428184766"/>
+        <c:axId val="1444187958"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1627451947"/>
+        <c:axId val="1428184766"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2076279430"/>
+        <c:crossAx val="1444187958"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2076279430"/>
+        <c:axId val="1444187958"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1627451947"/>
+        <c:crossAx val="1428184766"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1414164693"/>
-        <c:axId val="1405783839"/>
+        <c:axId val="1669809664"/>
+        <c:axId val="301631030"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1414164693"/>
+        <c:axId val="1669809664"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1405783839"/>
+        <c:crossAx val="301631030"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1405783839"/>
+        <c:axId val="301631030"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1414164693"/>
+        <c:crossAx val="1669809664"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1687,17 +1687,25 @@
       <c r="I10" s="7">
         <v>46240.0</v>
       </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="J10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L10" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M10" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N10" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O10" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11">
@@ -1737,7 +1745,7 @@
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
@@ -1777,7 +1785,7 @@
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13">
@@ -1817,7 +1825,7 @@
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14">
@@ -1857,7 +1865,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15">
@@ -1897,7 +1905,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16">
@@ -1937,7 +1945,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17">
@@ -1977,7 +1985,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18">
@@ -2017,7 +2025,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
@@ -2057,7 +2065,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20">
@@ -2097,7 +2105,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21">
@@ -2137,7 +2145,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Add report of 07/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,15 +24,6 @@
     <t>Module 1</t>
   </si>
   <si>
-    <t>Module 2</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
-  </si>
-  <si>
     <t>Découpe</t>
   </si>
   <si>
@@ -52,6 +43,15 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,7 +131,6 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -141,6 +140,7 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1428184766"/>
-        <c:axId val="1444187958"/>
+        <c:axId val="1000208090"/>
+        <c:axId val="2136916528"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1428184766"/>
+        <c:axId val="1000208090"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1444187958"/>
+        <c:crossAx val="2136916528"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1444187958"/>
+        <c:axId val="2136916528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1428184766"/>
+        <c:crossAx val="1000208090"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1669809664"/>
-        <c:axId val="301631030"/>
+        <c:axId val="1631075980"/>
+        <c:axId val="1971491981"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1669809664"/>
+        <c:axId val="1631075980"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="301631030"/>
+        <c:crossAx val="1971491981"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="301631030"/>
+        <c:axId val="1971491981"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1669809664"/>
+        <c:crossAx val="1631075980"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1233,63 +1233,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>46188.0</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>4.0</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="4">
         <v>3.0</v>
       </c>
-      <c r="D2" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E2" s="5">
+      <c r="D2" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="4">
         <v>0.0</v>
       </c>
       <c r="F2" s="6">
@@ -1300,19 +1300,19 @@
         <f t="shared" ref="G2:G21" si="2">SUM($F$2:F2)</f>
         <v>7</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="3">
         <v>46230.0</v>
       </c>
-      <c r="J2" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K2" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L2" s="5">
+      <c r="J2" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L2" s="4">
         <v>6.0</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="4">
         <v>1.0</v>
       </c>
       <c r="N2" s="6">
@@ -1325,19 +1325,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>46189.0</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="4">
         <v>2.0</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <v>5.0</v>
       </c>
-      <c r="D3" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E3" s="5">
+      <c r="D3" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E3" s="4">
         <v>0.0</v>
       </c>
       <c r="F3" s="6">
@@ -1348,19 +1348,19 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>46231.0</v>
       </c>
-      <c r="J3" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K3" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L3" s="5">
+      <c r="J3" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L3" s="4">
         <v>7.0</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3" s="4">
         <v>0.0</v>
       </c>
       <c r="N3" s="6">
@@ -1373,19 +1373,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>46190.0</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <v>2.0</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>5.0</v>
       </c>
-      <c r="D4" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E4" s="5">
+      <c r="D4" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="4">
         <v>0.0</v>
       </c>
       <c r="F4" s="6">
@@ -1396,19 +1396,19 @@
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>46232.0</v>
       </c>
-      <c r="J4" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K4" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L4" s="5">
+      <c r="J4" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L4" s="4">
         <v>7.0</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="4">
         <v>0.0</v>
       </c>
       <c r="N4" s="6">
@@ -1421,19 +1421,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>46191.0</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>4.0</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>3.0</v>
       </c>
-      <c r="D5" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E5" s="5">
+      <c r="D5" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E5" s="4">
         <v>0.0</v>
       </c>
       <c r="F5" s="6">
@@ -1444,19 +1444,19 @@
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="3">
         <v>46233.0</v>
       </c>
-      <c r="J5" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K5" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L5" s="5">
+      <c r="J5" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L5" s="4">
         <v>7.0</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="4">
         <v>0.0</v>
       </c>
       <c r="N5" s="6">
@@ -1469,19 +1469,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4">
+      <c r="A6" s="3">
         <v>46192.0</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="4">
         <v>1.0</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>6.0</v>
       </c>
-      <c r="D6" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E6" s="5">
+      <c r="D6" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="4">
         <v>0.0</v>
       </c>
       <c r="F6" s="6">
@@ -1492,19 +1492,19 @@
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="3">
         <v>46234.0</v>
       </c>
-      <c r="J6" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K6" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L6" s="5">
+      <c r="J6" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K6" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L6" s="4">
         <v>7.0</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="4">
         <v>0.0</v>
       </c>
       <c r="N6" s="6">
@@ -1520,16 +1520,16 @@
       <c r="A7" s="7">
         <v>46195.0</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="4">
         <v>3.0</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>3.0</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>1.0</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>0.0</v>
       </c>
       <c r="F7" s="6">
@@ -1543,16 +1543,16 @@
       <c r="I7" s="7">
         <v>46237.0</v>
       </c>
-      <c r="J7" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K7" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L7" s="5">
+      <c r="J7" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L7" s="4">
         <v>7.0</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="4">
         <v>0.0</v>
       </c>
       <c r="N7" s="6">
@@ -1568,16 +1568,16 @@
       <c r="A8" s="7">
         <v>46196.0</v>
       </c>
-      <c r="B8" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C8" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D8" s="5">
+      <c r="B8" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="4">
         <v>5.0</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <v>2.0</v>
       </c>
       <c r="F8" s="6">
@@ -1591,16 +1591,16 @@
       <c r="I8" s="7">
         <v>46238.0</v>
       </c>
-      <c r="J8" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K8" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L8" s="5">
+      <c r="J8" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K8" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L8" s="4">
         <v>7.0</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="4">
         <v>0.0</v>
       </c>
       <c r="N8" s="6">
@@ -1616,16 +1616,16 @@
       <c r="A9" s="7">
         <v>46197.0</v>
       </c>
-      <c r="B9" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C9" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D9" s="5">
+      <c r="B9" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="4">
         <v>5.0</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <v>2.0</v>
       </c>
       <c r="F9" s="6">
@@ -1639,16 +1639,16 @@
       <c r="I9" s="7">
         <v>46239.0</v>
       </c>
-      <c r="J9" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K9" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L9" s="5">
+      <c r="J9" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K9" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L9" s="4">
         <v>7.0</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="4">
         <v>0.0</v>
       </c>
       <c r="N9" s="6">
@@ -1664,16 +1664,16 @@
       <c r="A10" s="7">
         <v>46198.0</v>
       </c>
-      <c r="B10" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C10" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D10" s="5">
+      <c r="B10" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="4">
         <v>6.0</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <v>1.0</v>
       </c>
       <c r="F10" s="6">
@@ -1687,16 +1687,16 @@
       <c r="I10" s="7">
         <v>46240.0</v>
       </c>
-      <c r="J10" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="K10" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="L10" s="5">
+      <c r="J10" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K10" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L10" s="4">
         <v>7.0</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="4">
         <v>0.0</v>
       </c>
       <c r="N10" s="6">
@@ -1712,16 +1712,16 @@
       <c r="A11" s="7">
         <v>46199.0</v>
       </c>
-      <c r="B11" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C11" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D11" s="5">
+      <c r="B11" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="4">
         <v>6.0</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="4">
         <v>1.0</v>
       </c>
       <c r="F11" s="6">
@@ -1735,33 +1735,41 @@
       <c r="I11" s="7">
         <v>46241.0</v>
       </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="J11" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="K11" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="L11" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="M11" s="4">
+        <v>0.0</v>
+      </c>
       <c r="N11" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>46202.0</v>
       </c>
-      <c r="B12" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C12" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D12" s="5">
+      <c r="B12" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="4">
         <v>5.0</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <v>2.0</v>
       </c>
       <c r="F12" s="6">
@@ -1772,36 +1780,36 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>46244.0</v>
       </c>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
       <c r="N12" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>46203.0</v>
       </c>
-      <c r="B13" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C13" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D13" s="5">
+      <c r="B13" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="4">
         <v>7.0</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="4">
         <v>0.0</v>
       </c>
       <c r="F13" s="6">
@@ -1812,36 +1820,36 @@
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>46245.0</v>
       </c>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
       <c r="N13" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>46204.0</v>
       </c>
-      <c r="B14" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C14" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D14" s="5">
+      <c r="B14" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="4">
         <v>3.0</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="4">
         <v>4.0</v>
       </c>
       <c r="F14" s="6">
@@ -1852,36 +1860,36 @@
         <f t="shared" si="2"/>
         <v>91</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="3">
         <v>46246.0</v>
       </c>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
       <c r="N14" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>46205.0</v>
       </c>
-      <c r="B15" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C15" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D15" s="5">
+      <c r="B15" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D15" s="4">
         <v>5.0</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <v>2.0</v>
       </c>
       <c r="F15" s="6">
@@ -1892,36 +1900,36 @@
         <f t="shared" si="2"/>
         <v>98</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="3">
         <v>46247.0</v>
       </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
       <c r="N15" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>46206.0</v>
       </c>
-      <c r="B16" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C16" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D16" s="5">
+      <c r="B16" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C16" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D16" s="4">
         <v>7.0</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <v>0.0</v>
       </c>
       <c r="F16" s="6">
@@ -1932,36 +1940,36 @@
         <f t="shared" si="2"/>
         <v>105</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="3">
         <v>46248.0</v>
       </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
       <c r="N16" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7">
         <v>46209.0</v>
       </c>
-      <c r="B17" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C17" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D17" s="5">
+      <c r="B17" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C17" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D17" s="4">
         <v>7.0</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="4">
         <v>0.0</v>
       </c>
       <c r="F17" s="6">
@@ -1975,33 +1983,33 @@
       <c r="I17" s="7">
         <v>46251.0</v>
       </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
       <c r="N17" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7">
         <v>46210.0</v>
       </c>
-      <c r="B18" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C18" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D18" s="5">
+      <c r="B18" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C18" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D18" s="4">
         <v>7.0</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <v>0.0</v>
       </c>
       <c r="F18" s="6">
@@ -2015,33 +2023,33 @@
       <c r="I18" s="7">
         <v>46252.0</v>
       </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
       <c r="N18" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7">
         <v>46211.0</v>
       </c>
-      <c r="B19" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C19" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D19" s="5">
+      <c r="B19" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C19" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D19" s="4">
         <v>7.0</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="4">
         <v>0.0</v>
       </c>
       <c r="F19" s="6">
@@ -2055,33 +2063,33 @@
       <c r="I19" s="7">
         <v>46253.0</v>
       </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
       <c r="N19" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7">
         <v>46212.0</v>
       </c>
-      <c r="B20" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C20" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D20" s="5">
+      <c r="B20" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C20" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D20" s="4">
         <v>7.0</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="4">
         <v>0.0</v>
       </c>
       <c r="F20" s="6">
@@ -2095,33 +2103,33 @@
       <c r="I20" s="7">
         <v>46254.0</v>
       </c>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
       <c r="N20" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7">
         <v>46213.0</v>
       </c>
-      <c r="B21" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="C21" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="D21" s="5">
+      <c r="B21" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C21" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D21" s="4">
         <v>7.0</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="4">
         <v>0.0</v>
       </c>
       <c r="F21" s="6">
@@ -2135,17 +2143,17 @@
       <c r="I21" s="7">
         <v>46255.0</v>
       </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
       <c r="N21" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22">
@@ -2210,34 +2218,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="5">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2">
+        <v>11</v>
+      </c>
+      <c r="B4" s="5">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 10/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,6 +24,15 @@
     <t>Module 1</t>
   </si>
   <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
+  </si>
+  <si>
     <t>Découpe</t>
   </si>
   <si>
@@ -43,15 +52,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>Module 2</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,6 +131,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -140,7 +141,6 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1000208090"/>
-        <c:axId val="2136916528"/>
+        <c:axId val="1743724271"/>
+        <c:axId val="1566224433"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1000208090"/>
+        <c:axId val="1743724271"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2136916528"/>
+        <c:crossAx val="1566224433"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2136916528"/>
+        <c:axId val="1566224433"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1000208090"/>
+        <c:crossAx val="1743724271"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1631075980"/>
-        <c:axId val="1971491981"/>
+        <c:axId val="1891688965"/>
+        <c:axId val="289583430"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1631075980"/>
+        <c:axId val="1891688965"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1971491981"/>
+        <c:crossAx val="289583430"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1971491981"/>
+        <c:axId val="289583430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1631075980"/>
+        <c:crossAx val="1891688965"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1233,63 +1233,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="A1" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="F1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="O1" s="2" t="s">
+      <c r="K1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="M1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>46188.0</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="5">
         <v>4.0</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="5">
         <v>3.0</v>
       </c>
-      <c r="D2" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E2" s="4">
+      <c r="D2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0.0</v>
       </c>
       <c r="F2" s="6">
@@ -1300,19 +1300,19 @@
         <f t="shared" ref="G2:G21" si="2">SUM($F$2:F2)</f>
         <v>7</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="4">
         <v>46230.0</v>
       </c>
-      <c r="J2" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K2" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L2" s="4">
+      <c r="J2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K2" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L2" s="5">
         <v>6.0</v>
       </c>
-      <c r="M2" s="4">
+      <c r="M2" s="5">
         <v>1.0</v>
       </c>
       <c r="N2" s="6">
@@ -1325,19 +1325,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>46189.0</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="5">
         <v>2.0</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="5">
         <v>5.0</v>
       </c>
-      <c r="D3" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="D3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0.0</v>
       </c>
       <c r="F3" s="6">
@@ -1348,19 +1348,19 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="4">
         <v>46231.0</v>
       </c>
-      <c r="J3" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K3" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L3" s="4">
+      <c r="J3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K3" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L3" s="5">
         <v>7.0</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="5">
         <v>0.0</v>
       </c>
       <c r="N3" s="6">
@@ -1373,19 +1373,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>46190.0</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="5">
         <v>2.0</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="5">
         <v>5.0</v>
       </c>
-      <c r="D4" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E4" s="4">
+      <c r="D4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0.0</v>
       </c>
       <c r="F4" s="6">
@@ -1396,19 +1396,19 @@
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="4">
         <v>46232.0</v>
       </c>
-      <c r="J4" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K4" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L4" s="4">
+      <c r="J4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K4" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L4" s="5">
         <v>7.0</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="5">
         <v>0.0</v>
       </c>
       <c r="N4" s="6">
@@ -1421,19 +1421,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="4">
         <v>46191.0</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="5">
         <v>4.0</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="5">
         <v>3.0</v>
       </c>
-      <c r="D5" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E5" s="4">
+      <c r="D5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E5" s="5">
         <v>0.0</v>
       </c>
       <c r="F5" s="6">
@@ -1444,19 +1444,19 @@
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="4">
         <v>46233.0</v>
       </c>
-      <c r="J5" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K5" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L5" s="4">
+      <c r="J5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L5" s="5">
         <v>7.0</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="5">
         <v>0.0</v>
       </c>
       <c r="N5" s="6">
@@ -1469,19 +1469,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="4">
         <v>46192.0</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="5">
         <v>1.0</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="5">
         <v>6.0</v>
       </c>
-      <c r="D6" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E6" s="4">
+      <c r="D6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="5">
         <v>0.0</v>
       </c>
       <c r="F6" s="6">
@@ -1492,19 +1492,19 @@
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="4">
         <v>46234.0</v>
       </c>
-      <c r="J6" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K6" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L6" s="4">
+      <c r="J6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K6" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L6" s="5">
         <v>7.0</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>0.0</v>
       </c>
       <c r="N6" s="6">
@@ -1520,16 +1520,16 @@
       <c r="A7" s="7">
         <v>46195.0</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="5">
         <v>3.0</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="5">
         <v>3.0</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>1.0</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="5">
         <v>0.0</v>
       </c>
       <c r="F7" s="6">
@@ -1543,16 +1543,16 @@
       <c r="I7" s="7">
         <v>46237.0</v>
       </c>
-      <c r="J7" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K7" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L7" s="4">
+      <c r="J7" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L7" s="5">
         <v>7.0</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="5">
         <v>0.0</v>
       </c>
       <c r="N7" s="6">
@@ -1568,16 +1568,16 @@
       <c r="A8" s="7">
         <v>46196.0</v>
       </c>
-      <c r="B8" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D8" s="4">
+      <c r="B8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="5">
         <v>5.0</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="5">
         <v>2.0</v>
       </c>
       <c r="F8" s="6">
@@ -1591,16 +1591,16 @@
       <c r="I8" s="7">
         <v>46238.0</v>
       </c>
-      <c r="J8" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K8" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L8" s="4">
+      <c r="J8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K8" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L8" s="5">
         <v>7.0</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="5">
         <v>0.0</v>
       </c>
       <c r="N8" s="6">
@@ -1616,16 +1616,16 @@
       <c r="A9" s="7">
         <v>46197.0</v>
       </c>
-      <c r="B9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D9" s="4">
+      <c r="B9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="5">
         <v>5.0</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="5">
         <v>2.0</v>
       </c>
       <c r="F9" s="6">
@@ -1639,16 +1639,16 @@
       <c r="I9" s="7">
         <v>46239.0</v>
       </c>
-      <c r="J9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K9" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L9" s="4">
+      <c r="J9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K9" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L9" s="5">
         <v>7.0</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="5">
         <v>0.0</v>
       </c>
       <c r="N9" s="6">
@@ -1664,16 +1664,16 @@
       <c r="A10" s="7">
         <v>46198.0</v>
       </c>
-      <c r="B10" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D10" s="4">
+      <c r="B10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="5">
         <v>6.0</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="5">
         <v>1.0</v>
       </c>
       <c r="F10" s="6">
@@ -1687,16 +1687,16 @@
       <c r="I10" s="7">
         <v>46240.0</v>
       </c>
-      <c r="J10" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K10" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L10" s="4">
+      <c r="J10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L10" s="5">
         <v>7.0</v>
       </c>
-      <c r="M10" s="4">
+      <c r="M10" s="5">
         <v>0.0</v>
       </c>
       <c r="N10" s="6">
@@ -1712,16 +1712,16 @@
       <c r="A11" s="7">
         <v>46199.0</v>
       </c>
-      <c r="B11" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D11" s="4">
+      <c r="B11" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="5">
         <v>6.0</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="5">
         <v>1.0</v>
       </c>
       <c r="F11" s="6">
@@ -1735,16 +1735,16 @@
       <c r="I11" s="7">
         <v>46241.0</v>
       </c>
-      <c r="J11" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="K11" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="L11" s="4">
+      <c r="J11" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K11" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L11" s="5">
         <v>7.0</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M11" s="5">
         <v>0.0</v>
       </c>
       <c r="N11" s="6">
@@ -1757,19 +1757,19 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3">
+      <c r="A12" s="4">
         <v>46202.0</v>
       </c>
-      <c r="B12" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C12" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D12" s="4">
+      <c r="B12" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="5">
         <v>5.0</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="5">
         <v>2.0</v>
       </c>
       <c r="F12" s="6">
@@ -1780,36 +1780,44 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="4">
         <v>46244.0</v>
       </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
+      <c r="J12" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K12" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L12" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M12" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N12" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O12" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3">
+      <c r="A13" s="4">
         <v>46203.0</v>
       </c>
-      <c r="B13" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D13" s="4">
+      <c r="B13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="5">
         <v>7.0</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="5">
         <v>0.0</v>
       </c>
       <c r="F13" s="6">
@@ -1820,36 +1828,36 @@
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="4">
         <v>46245.0</v>
       </c>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
       <c r="N13" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3">
+      <c r="A14" s="4">
         <v>46204.0</v>
       </c>
-      <c r="B14" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D14" s="4">
+      <c r="B14" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="5">
         <v>3.0</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="5">
         <v>4.0</v>
       </c>
       <c r="F14" s="6">
@@ -1860,36 +1868,36 @@
         <f t="shared" si="2"/>
         <v>91</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="4">
         <v>46246.0</v>
       </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
       <c r="N14" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3">
+      <c r="A15" s="4">
         <v>46205.0</v>
       </c>
-      <c r="B15" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C15" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D15" s="4">
+      <c r="B15" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D15" s="5">
         <v>5.0</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="5">
         <v>2.0</v>
       </c>
       <c r="F15" s="6">
@@ -1900,36 +1908,36 @@
         <f t="shared" si="2"/>
         <v>98</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="4">
         <v>46247.0</v>
       </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
       <c r="N15" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3">
+      <c r="A16" s="4">
         <v>46206.0</v>
       </c>
-      <c r="B16" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C16" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D16" s="4">
+      <c r="B16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D16" s="5">
         <v>7.0</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="5">
         <v>0.0</v>
       </c>
       <c r="F16" s="6">
@@ -1940,36 +1948,36 @@
         <f t="shared" si="2"/>
         <v>105</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="4">
         <v>46248.0</v>
       </c>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
       <c r="N16" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7">
         <v>46209.0</v>
       </c>
-      <c r="B17" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C17" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D17" s="4">
+      <c r="B17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D17" s="5">
         <v>7.0</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="5">
         <v>0.0</v>
       </c>
       <c r="F17" s="6">
@@ -1983,33 +1991,33 @@
       <c r="I17" s="7">
         <v>46251.0</v>
       </c>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
       <c r="N17" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7">
         <v>46210.0</v>
       </c>
-      <c r="B18" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C18" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D18" s="4">
+      <c r="B18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D18" s="5">
         <v>7.0</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="5">
         <v>0.0</v>
       </c>
       <c r="F18" s="6">
@@ -2023,33 +2031,33 @@
       <c r="I18" s="7">
         <v>46252.0</v>
       </c>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
       <c r="N18" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7">
         <v>46211.0</v>
       </c>
-      <c r="B19" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C19" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D19" s="4">
+      <c r="B19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D19" s="5">
         <v>7.0</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="5">
         <v>0.0</v>
       </c>
       <c r="F19" s="6">
@@ -2063,33 +2071,33 @@
       <c r="I19" s="7">
         <v>46253.0</v>
       </c>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
       <c r="N19" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7">
         <v>46212.0</v>
       </c>
-      <c r="B20" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C20" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D20" s="4">
+      <c r="B20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D20" s="5">
         <v>7.0</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="5">
         <v>0.0</v>
       </c>
       <c r="F20" s="6">
@@ -2103,33 +2111,33 @@
       <c r="I20" s="7">
         <v>46254.0</v>
       </c>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
       <c r="N20" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7">
         <v>46213.0</v>
       </c>
-      <c r="B21" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="C21" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D21" s="4">
+      <c r="B21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="D21" s="5">
         <v>7.0</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="5">
         <v>0.0</v>
       </c>
       <c r="F21" s="6">
@@ -2143,17 +2151,17 @@
       <c r="I21" s="7">
         <v>46255.0</v>
       </c>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
       <c r="N21" s="6">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22">
@@ -2218,34 +2226,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="2">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="5">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="5">
+        <v>4</v>
+      </c>
+      <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="5">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 11/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -145,11 +145,11 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1743724271"/>
-        <c:axId val="1566224433"/>
+        <c:axId val="1055700549"/>
+        <c:axId val="891819412"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1743724271"/>
+        <c:axId val="1055700549"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1566224433"/>
+        <c:crossAx val="891819412"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1566224433"/>
+        <c:axId val="891819412"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1743724271"/>
+        <c:crossAx val="1055700549"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1891688965"/>
-        <c:axId val="289583430"/>
+        <c:axId val="1999216092"/>
+        <c:axId val="1474269497"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1891688965"/>
+        <c:axId val="1999216092"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="289583430"/>
+        <c:crossAx val="1474269497"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="289583430"/>
+        <c:axId val="1474269497"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1891688965"/>
+        <c:crossAx val="1999216092"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1831,17 +1831,25 @@
       <c r="I13" s="4">
         <v>46245.0</v>
       </c>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="J13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K13" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L13" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M13" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N13" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O13" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
@@ -1881,7 +1889,7 @@
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15">
@@ -1921,7 +1929,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
@@ -1961,7 +1969,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -2001,7 +2009,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18">
@@ -2041,7 +2049,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19">
@@ -2081,7 +2089,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20">
@@ -2121,7 +2129,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21">
@@ -2161,11 +2169,11 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22">
-      <c r="I22" s="9"/>
+      <c r="I22" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F21 N2:N21">
@@ -2195,7 +2203,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add report of 12/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1055700549"/>
-        <c:axId val="891819412"/>
+        <c:axId val="417506865"/>
+        <c:axId val="1534728290"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1055700549"/>
+        <c:axId val="417506865"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="891819412"/>
+        <c:crossAx val="1534728290"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="891819412"/>
+        <c:axId val="1534728290"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1055700549"/>
+        <c:crossAx val="417506865"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1999216092"/>
-        <c:axId val="1474269497"/>
+        <c:axId val="799636430"/>
+        <c:axId val="1812431230"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1999216092"/>
+        <c:axId val="799636430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1474269497"/>
+        <c:crossAx val="1812431230"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1474269497"/>
+        <c:axId val="1812431230"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1999216092"/>
+        <c:crossAx val="799636430"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1879,17 +1879,25 @@
       <c r="I14" s="4">
         <v>46246.0</v>
       </c>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="J14" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K14" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L14" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="M14" s="5">
+        <v>0.0</v>
+      </c>
       <c r="N14" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O14" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15">
@@ -1929,7 +1937,7 @@
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">
@@ -1969,7 +1977,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17">
@@ -2009,7 +2017,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18">
@@ -2049,7 +2057,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19">
@@ -2089,7 +2097,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20">
@@ -2129,7 +2137,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21">
@@ -2169,7 +2177,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Add report of 13/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="417506865"/>
-        <c:axId val="1534728290"/>
+        <c:axId val="1947020569"/>
+        <c:axId val="779744440"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="417506865"/>
+        <c:axId val="1947020569"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1534728290"/>
+        <c:crossAx val="779744440"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1534728290"/>
+        <c:axId val="779744440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="417506865"/>
+        <c:crossAx val="1947020569"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="799636430"/>
-        <c:axId val="1812431230"/>
+        <c:axId val="905990155"/>
+        <c:axId val="1316836362"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="799636430"/>
+        <c:axId val="905990155"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1812431230"/>
+        <c:crossAx val="1316836362"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1812431230"/>
+        <c:axId val="1316836362"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="799636430"/>
+        <c:crossAx val="905990155"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1927,17 +1927,25 @@
       <c r="I15" s="4">
         <v>46247.0</v>
       </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="J15" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K15" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L15" s="5">
+        <v>4.0</v>
+      </c>
+      <c r="M15" s="5">
+        <v>3.0</v>
+      </c>
       <c r="N15" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O15" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16">
@@ -1977,7 +1985,7 @@
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17">
@@ -2017,7 +2025,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18">
@@ -2057,7 +2065,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19">
@@ -2097,7 +2105,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20">
@@ -2137,7 +2145,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21">
@@ -2177,7 +2185,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Add report of 14/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1947020569"/>
-        <c:axId val="779744440"/>
+        <c:axId val="2099847580"/>
+        <c:axId val="1339636319"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1947020569"/>
+        <c:axId val="2099847580"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="779744440"/>
+        <c:crossAx val="1339636319"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="779744440"/>
+        <c:axId val="1339636319"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1947020569"/>
+        <c:crossAx val="2099847580"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="905990155"/>
-        <c:axId val="1316836362"/>
+        <c:axId val="1358390215"/>
+        <c:axId val="634241695"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="905990155"/>
+        <c:axId val="1358390215"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1316836362"/>
+        <c:crossAx val="634241695"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1316836362"/>
+        <c:axId val="634241695"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="905990155"/>
+        <c:crossAx val="1358390215"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1975,17 +1975,25 @@
       <c r="I16" s="4">
         <v>46248.0</v>
       </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+      <c r="J16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L16" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="M16" s="5">
+        <v>7.0</v>
+      </c>
       <c r="N16" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17">
@@ -2025,7 +2033,7 @@
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18">
@@ -2065,7 +2073,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19">
@@ -2105,7 +2113,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20">
@@ -2145,7 +2153,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21">
@@ -2185,7 +2193,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Add report of 17/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -27,13 +27,10 @@
     <t>Module 2</t>
   </si>
   <si>
-    <t>Module 3</t>
+    <t>Découpe</t>
   </si>
   <si>
-    <t>Module 4</t>
-  </si>
-  <si>
-    <t>Découpe</t>
+    <t>Module 3</t>
   </si>
   <si>
     <t>Extraction</t>
@@ -46,6 +43,9 @@
   </si>
   <si>
     <t>Total Jour</t>
+  </si>
+  <si>
+    <t>Module 4</t>
   </si>
   <si>
     <t>Progression Cumulée</t>
@@ -145,11 +145,11 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="2099847580"/>
-        <c:axId val="1339636319"/>
+        <c:axId val="226066591"/>
+        <c:axId val="1353538432"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2099847580"/>
+        <c:axId val="226066591"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1339636319"/>
+        <c:crossAx val="1353538432"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1339636319"/>
+        <c:axId val="1353538432"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2099847580"/>
+        <c:crossAx val="226066591"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="1358390215"/>
-        <c:axId val="634241695"/>
+        <c:axId val="560039780"/>
+        <c:axId val="1763549397"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1358390215"/>
+        <c:axId val="560039780"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="634241695"/>
+        <c:crossAx val="1763549397"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="634241695"/>
+        <c:axId val="1763549397"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1358390215"/>
+        <c:crossAx val="560039780"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1237,19 +1237,19 @@
         <v>0.0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>11</v>
@@ -1258,19 +1258,19 @@
         <v>12</v>
       </c>
       <c r="J1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="L1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="O1" s="3" t="s">
         <v>11</v>
@@ -2023,17 +2023,25 @@
       <c r="I17" s="7">
         <v>46251.0</v>
       </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+      <c r="J17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L17" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="M17" s="5">
+        <v>7.0</v>
+      </c>
       <c r="N17" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O17" s="6">
         <f t="shared" si="4"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18">
@@ -2073,7 +2081,7 @@
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19">
@@ -2113,7 +2121,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20">
@@ -2153,7 +2161,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21">
@@ -2193,11 +2201,11 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22">
-      <c r="I22" s="8"/>
+      <c r="I22" s="9"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F21 N2:N21">
@@ -2227,7 +2235,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2274,7 +2282,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
@@ -2283,7 +2291,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>

</xml_diff>

<commit_message>
Add report of 18/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,13 +24,7 @@
     <t>Module 1</t>
   </si>
   <si>
-    <t>Module 2</t>
-  </si>
-  <si>
     <t>Découpe</t>
-  </si>
-  <si>
-    <t>Module 3</t>
   </si>
   <si>
     <t>Extraction</t>
@@ -45,13 +39,19 @@
     <t>Total Jour</t>
   </si>
   <si>
-    <t>Module 4</t>
-  </si>
-  <si>
     <t>Progression Cumulée</t>
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -131,13 +131,13 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -145,11 +145,11 @@
     <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="226066591"/>
-        <c:axId val="1353538432"/>
+        <c:axId val="1247407353"/>
+        <c:axId val="221473016"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="226066591"/>
+        <c:axId val="1247407353"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1353538432"/>
+        <c:crossAx val="221473016"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1353538432"/>
+        <c:axId val="221473016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="226066591"/>
+        <c:crossAx val="1247407353"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="560039780"/>
-        <c:axId val="1763549397"/>
+        <c:axId val="2024021626"/>
+        <c:axId val="913399746"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="560039780"/>
+        <c:axId val="2024021626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1763549397"/>
+        <c:crossAx val="913399746"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1763549397"/>
+        <c:axId val="913399746"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="560039780"/>
+        <c:crossAx val="2024021626"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1233,51 +1233,51 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>46188.0</v>
       </c>
       <c r="B2" s="5">
@@ -1300,7 +1300,7 @@
         <f t="shared" ref="G2:G21" si="2">SUM($F$2:F2)</f>
         <v>7</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="3">
         <v>46230.0</v>
       </c>
       <c r="J2" s="5">
@@ -1325,7 +1325,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>46189.0</v>
       </c>
       <c r="B3" s="5">
@@ -1348,7 +1348,7 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>46231.0</v>
       </c>
       <c r="J3" s="5">
@@ -1373,7 +1373,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>46190.0</v>
       </c>
       <c r="B4" s="5">
@@ -1396,7 +1396,7 @@
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>46232.0</v>
       </c>
       <c r="J4" s="5">
@@ -1421,7 +1421,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>46191.0</v>
       </c>
       <c r="B5" s="5">
@@ -1444,7 +1444,7 @@
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="3">
         <v>46233.0</v>
       </c>
       <c r="J5" s="5">
@@ -1469,7 +1469,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4">
+      <c r="A6" s="3">
         <v>46192.0</v>
       </c>
       <c r="B6" s="5">
@@ -1492,7 +1492,7 @@
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="3">
         <v>46234.0</v>
       </c>
       <c r="J6" s="5">
@@ -1757,7 +1757,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>46202.0</v>
       </c>
       <c r="B12" s="5">
@@ -1780,7 +1780,7 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>46244.0</v>
       </c>
       <c r="J12" s="5">
@@ -1805,7 +1805,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>46203.0</v>
       </c>
       <c r="B13" s="5">
@@ -1828,7 +1828,7 @@
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>46245.0</v>
       </c>
       <c r="J13" s="5">
@@ -1853,7 +1853,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>46204.0</v>
       </c>
       <c r="B14" s="5">
@@ -1876,7 +1876,7 @@
         <f t="shared" si="2"/>
         <v>91</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="3">
         <v>46246.0</v>
       </c>
       <c r="J14" s="5">
@@ -1901,7 +1901,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>46205.0</v>
       </c>
       <c r="B15" s="5">
@@ -1924,7 +1924,7 @@
         <f t="shared" si="2"/>
         <v>98</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="3">
         <v>46247.0</v>
       </c>
       <c r="J15" s="5">
@@ -1949,7 +1949,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>46206.0</v>
       </c>
       <c r="B16" s="5">
@@ -1972,7 +1972,7 @@
         <f t="shared" si="2"/>
         <v>105</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="3">
         <v>46248.0</v>
       </c>
       <c r="J16" s="5">
@@ -2071,17 +2071,25 @@
       <c r="I18" s="7">
         <v>46252.0</v>
       </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="J18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L18" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="M18" s="5">
+        <v>7.0</v>
+      </c>
       <c r="N18" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O18" s="6">
         <f t="shared" si="4"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19">
@@ -2121,7 +2129,7 @@
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20">
@@ -2161,7 +2169,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21">
@@ -2201,11 +2209,11 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22">
-      <c r="I22" s="9"/>
+      <c r="I22" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F21 N2:N21">
@@ -2235,7 +2243,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2266,34 +2274,34 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2">
+        <v>11</v>
+      </c>
+      <c r="B4" s="4">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 19/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -24,6 +24,9 @@
     <t>Module 1</t>
   </si>
   <si>
+    <t>Module 2</t>
+  </si>
+  <si>
     <t>Découpe</t>
   </si>
   <si>
@@ -43,9 +46,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>Module 2</t>
   </si>
   <si>
     <t>Module 3</t>
@@ -131,13 +131,13 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1247407353"/>
-        <c:axId val="221473016"/>
+        <c:axId val="1205316964"/>
+        <c:axId val="1600925423"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1247407353"/>
+        <c:axId val="1205316964"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="221473016"/>
+        <c:crossAx val="1600925423"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="221473016"/>
+        <c:axId val="1600925423"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1247407353"/>
+        <c:crossAx val="1205316964"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="2024021626"/>
-        <c:axId val="913399746"/>
+        <c:axId val="261807921"/>
+        <c:axId val="2143686683"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2024021626"/>
+        <c:axId val="261807921"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="913399746"/>
+        <c:crossAx val="2143686683"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="913399746"/>
+        <c:axId val="2143686683"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2024021626"/>
+        <c:crossAx val="261807921"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1233,51 +1233,51 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="2" t="s">
+      <c r="I1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="O1" s="2" t="s">
+      <c r="M1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="O1" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>46188.0</v>
       </c>
       <c r="B2" s="5">
@@ -1300,7 +1300,7 @@
         <f t="shared" ref="G2:G21" si="2">SUM($F$2:F2)</f>
         <v>7</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="4">
         <v>46230.0</v>
       </c>
       <c r="J2" s="5">
@@ -1325,7 +1325,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>46189.0</v>
       </c>
       <c r="B3" s="5">
@@ -1348,7 +1348,7 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="4">
         <v>46231.0</v>
       </c>
       <c r="J3" s="5">
@@ -1373,7 +1373,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>46190.0</v>
       </c>
       <c r="B4" s="5">
@@ -1396,7 +1396,7 @@
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="4">
         <v>46232.0</v>
       </c>
       <c r="J4" s="5">
@@ -1421,7 +1421,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3">
+      <c r="A5" s="4">
         <v>46191.0</v>
       </c>
       <c r="B5" s="5">
@@ -1444,7 +1444,7 @@
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="4">
         <v>46233.0</v>
       </c>
       <c r="J5" s="5">
@@ -1469,7 +1469,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3">
+      <c r="A6" s="4">
         <v>46192.0</v>
       </c>
       <c r="B6" s="5">
@@ -1492,7 +1492,7 @@
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="4">
         <v>46234.0</v>
       </c>
       <c r="J6" s="5">
@@ -1757,7 +1757,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3">
+      <c r="A12" s="4">
         <v>46202.0</v>
       </c>
       <c r="B12" s="5">
@@ -1780,7 +1780,7 @@
         <f t="shared" si="2"/>
         <v>77</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="4">
         <v>46244.0</v>
       </c>
       <c r="J12" s="5">
@@ -1805,7 +1805,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3">
+      <c r="A13" s="4">
         <v>46203.0</v>
       </c>
       <c r="B13" s="5">
@@ -1828,7 +1828,7 @@
         <f t="shared" si="2"/>
         <v>84</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="4">
         <v>46245.0</v>
       </c>
       <c r="J13" s="5">
@@ -1853,7 +1853,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3">
+      <c r="A14" s="4">
         <v>46204.0</v>
       </c>
       <c r="B14" s="5">
@@ -1876,7 +1876,7 @@
         <f t="shared" si="2"/>
         <v>91</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="4">
         <v>46246.0</v>
       </c>
       <c r="J14" s="5">
@@ -1901,7 +1901,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3">
+      <c r="A15" s="4">
         <v>46205.0</v>
       </c>
       <c r="B15" s="5">
@@ -1924,7 +1924,7 @@
         <f t="shared" si="2"/>
         <v>98</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="4">
         <v>46247.0</v>
       </c>
       <c r="J15" s="5">
@@ -1949,7 +1949,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3">
+      <c r="A16" s="4">
         <v>46206.0</v>
       </c>
       <c r="B16" s="5">
@@ -1972,7 +1972,7 @@
         <f t="shared" si="2"/>
         <v>105</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="4">
         <v>46248.0</v>
       </c>
       <c r="J16" s="5">
@@ -2119,17 +2119,25 @@
       <c r="I19" s="7">
         <v>46253.0</v>
       </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
+      <c r="J19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L19" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="M19" s="5">
+        <v>7.0</v>
+      </c>
       <c r="N19" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O19" s="6">
         <f t="shared" si="4"/>
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
@@ -2169,7 +2177,7 @@
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21">
@@ -2209,7 +2217,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22">
@@ -2274,16 +2282,16 @@
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <f>SUM(Tracker!B2:B21)</f>
         <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="4">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
         <f>SUM(Tracker!C2:C21)</f>
         <v>25</v>
       </c>
@@ -2292,7 +2300,7 @@
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
         <v>85</v>
       </c>
@@ -2301,7 +2309,7 @@
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Add report of 20/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -27,6 +27,12 @@
     <t>Module 2</t>
   </si>
   <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>Module 4</t>
+  </si>
+  <si>
     <t>Découpe</t>
   </si>
   <si>
@@ -46,12 +52,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>Module 3</t>
-  </si>
-  <si>
-    <t>Module 4</t>
   </si>
   <si>
     <t>Tableau de Bord - Suivi des Modules</t>
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1205316964"/>
-        <c:axId val="1600925423"/>
+        <c:axId val="1492095998"/>
+        <c:axId val="249431380"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1205316964"/>
+        <c:axId val="1492095998"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1600925423"/>
+        <c:crossAx val="249431380"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1600925423"/>
+        <c:axId val="249431380"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1205316964"/>
+        <c:crossAx val="1492095998"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="261807921"/>
-        <c:axId val="2143686683"/>
+        <c:axId val="755505842"/>
+        <c:axId val="522031781"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="261807921"/>
+        <c:axId val="755505842"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2143686683"/>
+        <c:crossAx val="522031781"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2143686683"/>
+        <c:axId val="522031781"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="261807921"/>
+        <c:crossAx val="755505842"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1237,43 +1237,43 @@
         <v>0.0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="K1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="O1" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
@@ -2167,17 +2167,25 @@
       <c r="I20" s="7">
         <v>46254.0</v>
       </c>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="J20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L20" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="M20" s="5">
+        <v>7.0</v>
+      </c>
       <c r="N20" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O20" s="6">
         <f t="shared" si="4"/>
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21">
@@ -2217,7 +2225,7 @@
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22">
@@ -2298,7 +2306,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2">
         <f>SUM(Tracker!D2:D21)</f>
@@ -2307,7 +2315,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2">
         <f>SUM(Tracker!E2:E21)</f>

</xml_diff>

<commit_message>
Add report of 21/08
</commit_message>
<xml_diff>
--- a/specifications/TimeByModules.xlsx
+++ b/specifications/TimeByModules.xlsx
@@ -503,11 +503,11 @@
           </c:val>
         </c:ser>
         <c:overlap val="100"/>
-        <c:axId val="1492095998"/>
-        <c:axId val="249431380"/>
+        <c:axId val="1347218894"/>
+        <c:axId val="512330807"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1492095998"/>
+        <c:axId val="1347218894"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -563,10 +563,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="249431380"/>
+        <c:crossAx val="512330807"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="249431380"/>
+        <c:axId val="512330807"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -643,7 +643,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1492095998"/>
+        <c:crossAx val="1347218894"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -735,11 +735,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="755505842"/>
-        <c:axId val="522031781"/>
+        <c:axId val="429458529"/>
+        <c:axId val="1584738354"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="755505842"/>
+        <c:axId val="429458529"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -795,10 +795,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="522031781"/>
+        <c:crossAx val="1584738354"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="522031781"/>
+        <c:axId val="1584738354"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -875,7 +875,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="755505842"/>
+        <c:crossAx val="429458529"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2215,17 +2215,25 @@
       <c r="I21" s="7">
         <v>46255.0</v>
       </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
+      <c r="J21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="L21" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="M21" s="5">
+        <v>7.0</v>
+      </c>
       <c r="N21" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O21" s="6">
         <f t="shared" si="4"/>
-        <v>133</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22">

</xml_diff>